<commit_message>
Daily slate 2026-06-12 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-10.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-10.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E3" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F3" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G3" t="n">
-        <v>54.3</v>
+        <v>54.2</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F4" t="n">
         <v>43</v>
       </c>
       <c r="G4" t="n">
-        <v>47.6</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="5">
@@ -645,13 +645,13 @@
         <v>198</v>
       </c>
       <c r="E8" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F8" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G8" t="n">
-        <v>38.4</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="9">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1087</v>
+        <v>1122</v>
       </c>
       <c r="E11" t="n">
-        <v>692</v>
+        <v>717</v>
       </c>
       <c r="F11" t="n">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="G11" t="n">
-        <v>63.7</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="12">
@@ -816,13 +816,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E14" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F14" t="n">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="G14" t="n">
         <v>22.7</v>
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E15" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F15" t="n">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G15" t="n">
-        <v>15.3</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="16">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4551</v>
+        <v>4686</v>
       </c>
       <c r="E17" t="n">
-        <v>1042</v>
+        <v>1054</v>
       </c>
       <c r="F17" t="n">
-        <v>3509</v>
+        <v>3632</v>
       </c>
       <c r="G17" t="n">
-        <v>22.9</v>
+        <v>22.5</v>
       </c>
     </row>
   </sheetData>
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="Y4" t="n">
         <v>25</v>
@@ -1456,10 +1456,10 @@
         <v>180</v>
       </c>
       <c r="D7" t="n">
-        <v>63.7</v>
+        <v>63.9</v>
       </c>
       <c r="E7" t="n">
-        <v>1087</v>
+        <v>1122</v>
       </c>
       <c r="F7" t="n">
         <v>67.09999999999999</v>
@@ -1477,13 +1477,13 @@
         <v>22.7</v>
       </c>
       <c r="K7" t="n">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="L7" t="n">
-        <v>15.3</v>
+        <v>15.8</v>
       </c>
       <c r="M7" t="n">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="N7" t="n">
         <v>15.4</v>
@@ -1492,10 +1492,10 @@
         <v>65</v>
       </c>
       <c r="P7" t="n">
-        <v>22.9</v>
+        <v>22.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>4551</v>
+        <v>4686</v>
       </c>
       <c r="R7" t="n">
         <v>46.8</v>
@@ -1504,25 +1504,25 @@
         <v>77</v>
       </c>
       <c r="T7" t="n">
-        <v>47.6</v>
+        <v>48.2</v>
       </c>
       <c r="U7" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>38.4</v>
+        <v>39.4</v>
       </c>
       <c r="Y7" t="n">
         <v>198</v>
       </c>
       <c r="Z7" t="n">
-        <v>54.3</v>
+        <v>54.2</v>
       </c>
       <c r="AA7" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="AB7" t="n">
         <v>64.3</v>

</xml_diff>